<commit_message>
Refresh synthetic demo data
</commit_message>
<xml_diff>
--- a/data/outputs/ev_flex_daily_trading_report_sample.xlsx
+++ b/data/outputs/ev_flex_daily_trading_report_sample.xlsx
@@ -49,7 +49,7 @@
     <t>Generated at UTC</t>
   </si>
   <si>
-    <t>2026-08-31T14:33:08.054698+00:00</t>
+    <t>2026-09-07T13:06:49.621107+00:00</t>
   </si>
   <si>
     <t>Data status</t>
@@ -598,151 +598,151 @@
     <t>suggested_action</t>
   </si>
   <si>
-    <t>2026-08-31 14:33:06.251101+00:00</t>
-  </si>
-  <si>
-    <t>2026-08-31 14:33:06.281591+00:00</t>
-  </si>
-  <si>
-    <t>2026-08-31 14:33:06.305101+00:00</t>
-  </si>
-  <si>
-    <t>2026-08-31 14:33:06.338617+00:00</t>
-  </si>
-  <si>
-    <t>2026-08-31 14:33:06.369373+00:00</t>
-  </si>
-  <si>
-    <t>2026-08-31 14:33:06.394536+00:00</t>
-  </si>
-  <si>
-    <t>2026-08-31 14:33:06.413569+00:00</t>
-  </si>
-  <si>
-    <t>2026-08-31 14:33:06.440459+00:00</t>
-  </si>
-  <si>
-    <t>2026-08-31 14:33:06.459630+00:00</t>
-  </si>
-  <si>
-    <t>2026-08-31 14:33:06.481219+00:00</t>
-  </si>
-  <si>
-    <t>2026-08-31 14:33:06.505419+00:00</t>
-  </si>
-  <si>
-    <t>2026-08-31 14:33:06.531867+00:00</t>
-  </si>
-  <si>
-    <t>2026-08-31 14:33:06.552440+00:00</t>
-  </si>
-  <si>
-    <t>2026-08-31 14:33:06.577921+00:00</t>
-  </si>
-  <si>
-    <t>2026-08-31 14:33:06.596703+00:00</t>
-  </si>
-  <si>
-    <t>2026-08-31 14:33:06.615743+00:00</t>
-  </si>
-  <si>
-    <t>2026-08-31 14:33:06.632319+00:00</t>
-  </si>
-  <si>
-    <t>2026-08-31 14:33:06.651255+00:00</t>
-  </si>
-  <si>
-    <t>2026-08-31 14:33:06.676173+00:00</t>
-  </si>
-  <si>
-    <t>2026-08-31 14:33:06.701457+00:00</t>
-  </si>
-  <si>
-    <t>2026-08-31 14:33:06.719376+00:00</t>
-  </si>
-  <si>
-    <t>2026-08-31 14:33:06.732804+00:00</t>
-  </si>
-  <si>
-    <t>2026-08-31 14:33:06.746638+00:00</t>
-  </si>
-  <si>
-    <t>2026-08-31 14:33:06.765007+00:00</t>
-  </si>
-  <si>
-    <t>2026-08-31 14:33:06.817752+00:00</t>
-  </si>
-  <si>
-    <t>2026-08-31 14:33:06.878504+00:00</t>
-  </si>
-  <si>
-    <t>2026-08-31 14:33:06.901414+00:00</t>
-  </si>
-  <si>
-    <t>2026-08-31 14:33:06.934066+00:00</t>
-  </si>
-  <si>
-    <t>2026-08-31 14:33:06.961739+00:00</t>
-  </si>
-  <si>
-    <t>2026-08-31 14:33:06.986898+00:00</t>
-  </si>
-  <si>
-    <t>2026-08-31 14:33:07.005564+00:00</t>
-  </si>
-  <si>
-    <t>2026-08-31 14:33:07.032351+00:00</t>
-  </si>
-  <si>
-    <t>2026-08-31 14:33:07.051491+00:00</t>
-  </si>
-  <si>
-    <t>2026-08-31 14:33:07.073137+00:00</t>
-  </si>
-  <si>
-    <t>2026-08-31 14:33:07.097518+00:00</t>
-  </si>
-  <si>
-    <t>2026-08-31 14:33:07.123932+00:00</t>
-  </si>
-  <si>
-    <t>2026-08-31 14:33:07.144175+00:00</t>
-  </si>
-  <si>
-    <t>2026-08-31 14:33:07.169969+00:00</t>
-  </si>
-  <si>
-    <t>2026-08-31 14:33:07.188778+00:00</t>
-  </si>
-  <si>
-    <t>2026-08-31 14:33:07.207735+00:00</t>
-  </si>
-  <si>
-    <t>2026-08-31 14:33:07.224391+00:00</t>
-  </si>
-  <si>
-    <t>2026-08-31 14:33:07.243226+00:00</t>
-  </si>
-  <si>
-    <t>2026-08-31 14:33:07.268385+00:00</t>
-  </si>
-  <si>
-    <t>2026-08-31 14:33:07.293986+00:00</t>
-  </si>
-  <si>
-    <t>2026-08-31 14:33:07.311675+00:00</t>
-  </si>
-  <si>
-    <t>2026-08-31 14:33:07.325288+00:00</t>
-  </si>
-  <si>
-    <t>2026-08-31 14:33:07.338957+00:00</t>
-  </si>
-  <si>
-    <t>2026-08-31 14:33:07.357447+00:00</t>
-  </si>
-  <si>
-    <t>2026-08-31 14:33:07.489763+00:00</t>
+    <t>2026-09-07 13:06:47.791752+00:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 13:06:47.824756+00:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 13:06:47.851543+00:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 13:06:47.889280+00:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 13:06:47.921706+00:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 13:06:47.948874+00:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 13:06:47.968851+00:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 13:06:47.997824+00:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 13:06:48.018384+00:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 13:06:48.041921+00:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 13:06:48.068182+00:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 13:06:48.096465+00:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 13:06:48.118449+00:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 13:06:48.146125+00:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 13:06:48.166353+00:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 13:06:48.187008+00:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 13:06:48.204865+00:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 13:06:48.225228+00:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 13:06:48.252123+00:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 13:06:48.279854+00:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 13:06:48.299452+00:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 13:06:48.314164+00:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 13:06:48.329089+00:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 13:06:48.349210+00:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 13:06:48.405933+00:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 13:06:48.458216+00:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 13:06:48.482859+00:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 13:06:48.518256+00:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 13:06:48.548360+00:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 13:06:48.575662+00:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 13:06:48.595788+00:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 13:06:48.624649+00:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 13:06:48.645138+00:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 13:06:48.668478+00:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 13:06:48.694886+00:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 13:06:48.723584+00:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 13:06:48.745600+00:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 13:06:48.773461+00:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 13:06:48.793658+00:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 13:06:48.814212+00:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 13:06:48.832022+00:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 13:06:48.852519+00:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 13:06:48.879830+00:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 13:06:48.907183+00:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 13:06:48.926496+00:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 13:06:48.941380+00:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 13:06:48.956293+00:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 13:06:48.976314+00:00</t>
+  </si>
+  <si>
+    <t>2026-09-07 13:06:49.116804+00:00</t>
   </si>
   <si>
     <t>low</t>
@@ -1330,7 +1330,7 @@
     <t>MWh</t>
   </si>
   <si>
-    <t>2026-08-31T14:33:01.574773+00:00</t>
+    <t>2026-09-07T13:06:43.002543+00:00</t>
   </si>
   <si>
     <t>synthetic scenario: base</t>

</xml_diff>